<commit_message>
feat: implement spatial function checks, add evaluation scripts, and update model benchmarks.
</commit_message>
<xml_diff>
--- a/evals/audio/seamless/eval_results_seamless_pipeline.xlsx
+++ b/evals/audio/seamless/eval_results_seamless_pipeline.xlsx
@@ -569,7 +569,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>कैफे या रेस्टोरेंट खोजें।</t>
+          <t>Find cafes or restaurants.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>कॅफे किंवा रेस्टॉरंट शोधा.</t>
+          <t>Find cafes or restaurants.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -663,7 +663,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>కేఫ్‌లు లేదా రెస్టారెంట్‌లను కనుగొనండి.</t>
+          <t>Find cafes or restaurants.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -672,7 +672,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>கஃபேக்கள் அல்லது உணவகங்களை கண்டுபிடி.</t>
+          <t>Find cafes or restaurants.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -719,7 +719,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>cafe ya restaurant dhundho.</t>
+          <t>Find cafes or restaurants.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>koi khane peene ki jagah batao, cafe waghera</t>
+          <t>Find cafes or restaurants.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.875</v>
+        <v>2.25</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="9">
@@ -851,7 +851,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ਕੈਫੇ ਜਾਂ ਰੈਸਟੋਰੈਂਟ ਲੱਭੋ।</t>
+          <t>Find cafes or restaurants.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>क्या कोई कैफे 24/7 खुला है?</t>
+          <t>Are there any cafes open 24/7?</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1.333333333333333</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -992,7 +992,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>कोणते कॅफे २४/७ उघडे आहे का?</t>
+          <t>Are there any cafes open 24/7?</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ఏదైనా కేఫ్ 24/7 తెరిచి ఉందా?</t>
+          <t>Are there any cafes open 24/7?</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1.2</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>0.667</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="14">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ஏதாவது கஃபே 24/7 திறந்திருக்கிறதா?</t>
+          <t>Are there any cafes open 24/7?</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>koi cafe 24/7 khula hai kya?</t>
+          <t>Are there any cafes open 24/7?</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1.166666666666667</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>koi cafe hai kya jo din raat khula rehta hai?</t>
+          <t>Are there any cafes open 24/7?</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>1.166666666666667</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ਕੀ ਇੱਥੇ ਕੋਈ ਕੈਫੇ 24/7 ਖੁੱਲ੍ਹੇ ਹਨ?</t>
+          <t>Are there any cafes open 24/7?</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>मैं बहुत तनाव में हूँ, मुझे शांत जगह कहाँ मिलेगी?</t>
+          <t>I am so stressed, where can I find a calm place?</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1330,7 +1330,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.1</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>मी खूप तणावात आहे, मला शांत जागा कुठे मिळेल?</t>
+          <t>I am so stressed, where can I find a calm place?</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.111111111111111</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>నేను చాలా ఒత్తిడిలో ఉన్నాను, ప్రశాంతమైన ప్రదేశం ఎక్కడ దొరుకుతుంది?</t>
+          <t>I am so stressed, where can I find a calm place?</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.625</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>நான் மிகவும் மன அழுத்தத்தில் இருக்கிறேன், அமைதியான இடம் எங்கே கிடைக்கும்?</t>
+          <t>I am so stressed, where can I find a calm place?</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1.111111111111111</v>
+        <v>0.3636363636363636</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>main bahut stressed hoon, koi shant jagah kahan milegi?</t>
+          <t>I am so stressed, where can I find a calm place?</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1.222222222222222</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>yaar dimaag kharab ho raha hai, koi shanti wali jagah bata de</t>
+          <t>I am so stressed, where can I find a calm place?</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ਮੈਂ ਬਹੁਤ ਤਣਾਅ ਵਿੱਚ ਹਾਂ, ਮੈਨੂੰ ਇੱਕ ਸ਼ਾਂਤ ਜਗ੍ਹਾ ਕਿੱਥੇ ਮਿਲ ਸਕਦੀ ਹੈ?</t>
+          <t>I am so stressed, where can I find a calm place?</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
         <v>0.4615384615384615</v>
       </c>
       <c r="K26" t="n">
-        <v>0.667</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="27">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>छात्रावास के सबसे करीब कैफे खोजें।</t>
+          <t>Find the nearest cafe to the dormitory.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1706,7 +1706,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1.166666666666667</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
         <v>0.5714285714285715</v>
       </c>
       <c r="K27" t="n">
-        <v>0.667</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="28">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>वसतिगृहाच्या सर्वात जवळचा कॅफे शोधा.</t>
+          <t>Find the nearest cafe to the dormitory.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1.4</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1772,7 +1772,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="K28" t="n">
-        <v>0.667</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="29">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>హాస్టల్‌కు అత్యంత సమీపంలో ఉన్న కేఫ్‌ని కనుగొనండి.</t>
+          <t>Find the nearest cafe to the dormitory.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1800,7 +1800,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1.166666666666667</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>விடுதிக்கு மிக அருகில் உள்ள கஃபேவை கண்டுபிடி.</t>
+          <t>Find the nearest cafe to the dormitory.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1847,7 +1847,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1.166666666666667</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1866,7 +1866,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
-        <v>0.333</v>
+        <v>0.286</v>
       </c>
     </row>
     <row r="31">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>hostel ke sabse paas wala cafe batao.</t>
+          <t>Find the nearest cafe to the dormitory.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1894,7 +1894,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1.142857142857143</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         <v>0.5714285714285715</v>
       </c>
       <c r="K31" t="n">
-        <v>0.667</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="32">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>hostel ke nazdeek sabse paas wali tapri kidhar hai?</t>
+          <t>Find the nearest cafe to the dormitory.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1941,7 +1941,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1960,7 +1960,7 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>0.667</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="33">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ਡਾਰਮਿਟਰੀ ਲਈ ਨਜ਼ਦੀਕੀ ਕੈਫੇ ਲੱਭੋ.</t>
+          <t>Find the nearest cafe to the dormitory.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1988,7 +1988,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1.2</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2007,7 +2007,7 @@
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>0.167</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="34">
@@ -2054,7 +2054,7 @@
         <v>0.2352941176470588</v>
       </c>
       <c r="K34" t="n">
-        <v>0.667</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="35">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ऐसा पुस्तकालय खोजें जो स्कूल नहीं है।</t>
+          <t>Find a library that is NOT a school.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2082,7 +2082,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1.142857142857143</v>
+        <v>0.125</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
         <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>0.667</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="36">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>शाळा नसलेले ग्रंथालय शोधा.</t>
+          <t>Find a library that is NOT a school.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2129,7 +2129,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
+        <v>0.75</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>0.667</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="37">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>పాఠశాల కాని లైబ్రరీని కనుగొనండి.</t>
+          <t>Find a library that is NOT a school.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2176,7 +2176,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>1.5</v>
+        <v>0.625</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>பள்ளி அல்லாத நூலகத்தை கண்டுபிடி.</t>
+          <t>Find a library that is NOT a school.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>0.125</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
         <v>1</v>
       </c>
       <c r="K38" t="n">
-        <v>0.667</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="39">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>library dhundho jo school nahi hai.</t>
+          <t>Find a library that is NOT a school.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2270,7 +2270,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>1.166666666666667</v>
+        <v>0.125</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2289,7 +2289,7 @@
         <v>0.2352941176470588</v>
       </c>
       <c r="K39" t="n">
-        <v>0.667</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="40">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>bhai ek library chahiye but school nahi honi chahiye.</t>
+          <t>Find a library that is NOT a school.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>0.625</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ਅਜਿਹੀ ਲਾਇਬ੍ਰੇਰੀ ਲੱਭੋ ਜੋ ਸਕੂਲ ਨਾ ਹੋਵੇ।</t>
+          <t>Find a library that is NOT a school.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2364,7 +2364,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1.571428571428571</v>
+        <v>1.375</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -2383,7 +2383,7 @@
         <v>0.4545454545454545</v>
       </c>
       <c r="K41" t="n">
-        <v>0.667</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="42">
@@ -2430,7 +2430,7 @@
         <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="43">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>लाइब्रेरी कहाँ है?</t>
+          <t>Where is the library?</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>1.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2477,7 +2477,7 @@
         <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="44">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ग्रंथालय कुठे आहे?</t>
+          <t>Where is the library?</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2524,7 +2524,7 @@
         <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="45">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>లైబ్రరీ ఎక్కడ ఉంది?</t>
+          <t>Where is the library?</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2571,7 +2571,7 @@
         <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="46">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>நூலகம் எங்கே இருக்கிறது?</t>
+          <t>Where is the library?</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2618,7 +2618,7 @@
         <v>1</v>
       </c>
       <c r="K46" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="47">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>library kahan hai?</t>
+          <t>Where is the library?</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2646,7 +2646,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2665,7 +2665,7 @@
         <v>1</v>
       </c>
       <c r="K47" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="48">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>bhai campus me library kidhar milegi?</t>
+          <t>Where is the library?</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2693,7 +2693,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ਲਾਇਬ੍ਰੇਰੀ ਕਿੱਥੇ ਹੈ?</t>
+          <t>Where is the library?</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>1.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2759,7 +2759,7 @@
         <v>1</v>
       </c>
       <c r="K49" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="50">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>लाइब्रेरी के 500 मीटर के भीतर एक कैफे खोजें।</t>
+          <t>Find a cafe within 500 meters of the library.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2834,7 +2834,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ग्रंथालयाच्या ५०० मीटर अंतरावर कॅफे शोधा.</t>
+          <t>Find a cafe within 500 meters of the library.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>లైబ్రరీకి 500 మీటర్ల లోపు కేఫ్‌ని కనుగొనండి.</t>
+          <t>Find a cafe within 500 meters of the library.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2928,7 +2928,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1.666666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>நூலகத்தின் 500 மீட்டருக்குள் ஒரு கஃபேவை கண்டுபிடி.</t>
+          <t>Find a cafe within 500 meters of the library.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2975,7 +2975,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>1.666666666666667</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>library ke 500 meter ke andar ek cafe batao.</t>
+          <t>Find a cafe within 500 meters of the library.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>1.111111111111111</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>library ke aas paas 500m me koi chai ki tapri hai kya?</t>
+          <t>Find a cafe within 500 meters of the library.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>1</v>
+        <v>1.111111111111111</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ਲਾਇਬ੍ਰੇਰੀ ਦੇ 500 ਮੀਟਰ ਦੇ ਅੰਦਰ ਇੱਕ ਕੈਫੇ ਲੱਭੋ।</t>
+          <t>Find a cafe within 500 meters of the library.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3116,7 +3116,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>1.111111111111111</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>

</xml_diff>